<commit_message>
Trying to add gitnore files
</commit_message>
<xml_diff>
--- a/logs/grind_stats.xlsx
+++ b/logs/grind_stats.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S97"/>
+  <dimension ref="A1:S118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6371,6 +6371,1287 @@
         <v>0</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:14:09</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>731</v>
+      </c>
+      <c r="C98" t="n">
+        <v>12860</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
+        <v>2038</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
+        <v>17289</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>4657</v>
+      </c>
+      <c r="K98" t="n">
+        <v>16154</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" t="n">
+        <v>155</v>
+      </c>
+      <c r="P98" t="n">
+        <v>176</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>23094</v>
+      </c>
+      <c r="R98" t="n">
+        <v>296</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:23:08</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4816</v>
+      </c>
+      <c r="C99" t="n">
+        <v>15774</v>
+      </c>
+      <c r="D99" t="n">
+        <v>461</v>
+      </c>
+      <c r="E99" t="n">
+        <v>2537</v>
+      </c>
+      <c r="F99" t="n">
+        <v>488</v>
+      </c>
+      <c r="G99" t="n">
+        <v>17289</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>292</v>
+      </c>
+      <c r="J99" t="n">
+        <v>5071</v>
+      </c>
+      <c r="K99" t="n">
+        <v>16154</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
+        <v>0</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" t="n">
+        <v>156</v>
+      </c>
+      <c r="P99" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>145406</v>
+      </c>
+      <c r="R99" t="n">
+        <v>296</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:56:09</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>5982</v>
+      </c>
+      <c r="C100" t="n">
+        <v>18729</v>
+      </c>
+      <c r="D100" t="n">
+        <v>2222</v>
+      </c>
+      <c r="E100" t="n">
+        <v>4478</v>
+      </c>
+      <c r="F100" t="n">
+        <v>2592</v>
+      </c>
+      <c r="G100" t="n">
+        <v>17604</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="n">
+        <v>999</v>
+      </c>
+      <c r="J100" t="n">
+        <v>7592</v>
+      </c>
+      <c r="K100" t="n">
+        <v>16154</v>
+      </c>
+      <c r="L100" t="n">
+        <v>215</v>
+      </c>
+      <c r="M100" t="n">
+        <v>0</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" t="n">
+        <v>156</v>
+      </c>
+      <c r="P100" t="n">
+        <v>181</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
+        <v>296</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-03-01 21:18:37</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>10207</v>
+      </c>
+      <c r="C101" t="n">
+        <v>40624</v>
+      </c>
+      <c r="D101" t="n">
+        <v>2535</v>
+      </c>
+      <c r="E101" t="n">
+        <v>9214</v>
+      </c>
+      <c r="F101" t="n">
+        <v>3128</v>
+      </c>
+      <c r="G101" t="n">
+        <v>43280</v>
+      </c>
+      <c r="H101" t="n">
+        <v>19</v>
+      </c>
+      <c r="I101" t="n">
+        <v>1795</v>
+      </c>
+      <c r="J101" t="n">
+        <v>17101</v>
+      </c>
+      <c r="K101" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L101" t="n">
+        <v>349</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" t="n">
+        <v>97</v>
+      </c>
+      <c r="O101" t="n">
+        <v>157</v>
+      </c>
+      <c r="P101" t="n">
+        <v>184</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>358813</v>
+      </c>
+      <c r="R101" t="n">
+        <v>296</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-03-01 21:26:32</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>13284</v>
+      </c>
+      <c r="C102" t="n">
+        <v>46022</v>
+      </c>
+      <c r="D102" t="n">
+        <v>3413</v>
+      </c>
+      <c r="E102" t="n">
+        <v>11531</v>
+      </c>
+      <c r="F102" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>28</v>
+      </c>
+      <c r="I102" t="n">
+        <v>2689</v>
+      </c>
+      <c r="J102" t="n">
+        <v>19563</v>
+      </c>
+      <c r="K102" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L102" t="n">
+        <v>574</v>
+      </c>
+      <c r="M102" t="n">
+        <v>0</v>
+      </c>
+      <c r="N102" t="n">
+        <v>160</v>
+      </c>
+      <c r="O102" t="n">
+        <v>160</v>
+      </c>
+      <c r="P102" t="n">
+        <v>185</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>464318</v>
+      </c>
+      <c r="R102" t="n">
+        <v>296</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-03-01 22:29:27</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>16528</v>
+      </c>
+      <c r="C103" t="n">
+        <v>49565</v>
+      </c>
+      <c r="D103" t="n">
+        <v>4554</v>
+      </c>
+      <c r="E103" t="n">
+        <v>13094</v>
+      </c>
+      <c r="F103" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G103" t="n">
+        <v>44708</v>
+      </c>
+      <c r="H103" t="n">
+        <v>28</v>
+      </c>
+      <c r="I103" t="n">
+        <v>3406</v>
+      </c>
+      <c r="J103" t="n">
+        <v>22514</v>
+      </c>
+      <c r="K103" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L103" t="n">
+        <v>650</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="n">
+        <v>162</v>
+      </c>
+      <c r="P103" t="n">
+        <v>186</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>616799</v>
+      </c>
+      <c r="R103" t="n">
+        <v>296</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-03-01 22:33:57</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>19459</v>
+      </c>
+      <c r="C104" t="n">
+        <v>53183</v>
+      </c>
+      <c r="D104" t="n">
+        <v>5765</v>
+      </c>
+      <c r="E104" t="n">
+        <v>15861</v>
+      </c>
+      <c r="F104" t="n">
+        <v>7028</v>
+      </c>
+      <c r="G104" t="n">
+        <v>45029</v>
+      </c>
+      <c r="H104" t="n">
+        <v>40</v>
+      </c>
+      <c r="I104" t="n">
+        <v>4505</v>
+      </c>
+      <c r="J104" t="n">
+        <v>25634</v>
+      </c>
+      <c r="K104" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L104" t="n">
+        <v>1142</v>
+      </c>
+      <c r="M104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
+        <v>163</v>
+      </c>
+      <c r="P104" t="n">
+        <v>187</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>657569</v>
+      </c>
+      <c r="R104" t="n">
+        <v>296</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-03-01 22:42:40</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>25142</v>
+      </c>
+      <c r="C105" t="n">
+        <v>57093</v>
+      </c>
+      <c r="D105" t="n">
+        <v>6745</v>
+      </c>
+      <c r="E105" t="n">
+        <v>17875</v>
+      </c>
+      <c r="F105" t="n">
+        <v>7894</v>
+      </c>
+      <c r="G105" t="n">
+        <v>45709</v>
+      </c>
+      <c r="H105" t="n">
+        <v>45</v>
+      </c>
+      <c r="I105" t="n">
+        <v>5017</v>
+      </c>
+      <c r="J105" t="n">
+        <v>26797</v>
+      </c>
+      <c r="K105" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L105" t="n">
+        <v>1289</v>
+      </c>
+      <c r="M105" t="n">
+        <v>0</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>163</v>
+      </c>
+      <c r="P105" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>788160</v>
+      </c>
+      <c r="R105" t="n">
+        <v>296</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:09:57</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>28537</v>
+      </c>
+      <c r="C106" t="n">
+        <v>60786</v>
+      </c>
+      <c r="D106" t="n">
+        <v>8184</v>
+      </c>
+      <c r="E106" t="n">
+        <v>20210</v>
+      </c>
+      <c r="F106" t="n">
+        <v>9609</v>
+      </c>
+      <c r="G106" t="n">
+        <v>46850</v>
+      </c>
+      <c r="H106" t="n">
+        <v>53</v>
+      </c>
+      <c r="I106" t="n">
+        <v>6070</v>
+      </c>
+      <c r="J106" t="n">
+        <v>29720</v>
+      </c>
+      <c r="K106" t="n">
+        <v>39815</v>
+      </c>
+      <c r="L106" t="n">
+        <v>1470</v>
+      </c>
+      <c r="M106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
+        <v>163</v>
+      </c>
+      <c r="P106" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>840197</v>
+      </c>
+      <c r="R106" t="n">
+        <v>296</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:18:55</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>32418</v>
+      </c>
+      <c r="C107" t="n">
+        <v>64347</v>
+      </c>
+      <c r="D107" t="n">
+        <v>9221</v>
+      </c>
+      <c r="E107" t="n">
+        <v>21759</v>
+      </c>
+      <c r="F107" t="n">
+        <v>10927</v>
+      </c>
+      <c r="G107" t="n">
+        <v>47533</v>
+      </c>
+      <c r="H107" t="n">
+        <v>60</v>
+      </c>
+      <c r="I107" t="n">
+        <v>7055</v>
+      </c>
+      <c r="J107" t="n">
+        <v>31955</v>
+      </c>
+      <c r="K107" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L107" t="n">
+        <v>1568</v>
+      </c>
+      <c r="M107" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="n">
+        <v>164</v>
+      </c>
+      <c r="P107" t="n">
+        <v>192</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>941321</v>
+      </c>
+      <c r="R107" t="n">
+        <v>296</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-03-02 14:51:51</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>35939</v>
+      </c>
+      <c r="C108" t="n">
+        <v>70003</v>
+      </c>
+      <c r="D108" t="n">
+        <v>11174</v>
+      </c>
+      <c r="E108" t="n">
+        <v>23612</v>
+      </c>
+      <c r="F108" t="n">
+        <v>13117</v>
+      </c>
+      <c r="G108" t="n">
+        <v>48336</v>
+      </c>
+      <c r="H108" t="n">
+        <v>78</v>
+      </c>
+      <c r="I108" t="n">
+        <v>7802</v>
+      </c>
+      <c r="J108" t="n">
+        <v>34292</v>
+      </c>
+      <c r="K108" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L108" t="n">
+        <v>1866</v>
+      </c>
+      <c r="M108" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>167</v>
+      </c>
+      <c r="P108" t="n">
+        <v>194</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>296</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-03-02 15:22:09</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>37568</v>
+      </c>
+      <c r="C109" t="n">
+        <v>73544</v>
+      </c>
+      <c r="D109" t="n">
+        <v>12578</v>
+      </c>
+      <c r="E109" t="n">
+        <v>24885</v>
+      </c>
+      <c r="F109" t="n">
+        <v>14597</v>
+      </c>
+      <c r="G109" t="n">
+        <v>49043</v>
+      </c>
+      <c r="H109" t="n">
+        <v>97</v>
+      </c>
+      <c r="I109" t="n">
+        <v>8708</v>
+      </c>
+      <c r="J109" t="n">
+        <v>37141</v>
+      </c>
+      <c r="K109" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L109" t="n">
+        <v>2011</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>170</v>
+      </c>
+      <c r="P109" t="n">
+        <v>194</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>1142734</v>
+      </c>
+      <c r="R109" t="n">
+        <v>296</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-03-02 15:30:35</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>40605</v>
+      </c>
+      <c r="C110" t="n">
+        <v>78429</v>
+      </c>
+      <c r="D110" t="n">
+        <v>13146</v>
+      </c>
+      <c r="E110" t="n">
+        <v>26174</v>
+      </c>
+      <c r="F110" t="n">
+        <v>15450</v>
+      </c>
+      <c r="G110" t="n">
+        <v>49369</v>
+      </c>
+      <c r="H110" t="n">
+        <v>111</v>
+      </c>
+      <c r="I110" t="n">
+        <v>9521</v>
+      </c>
+      <c r="J110" t="n">
+        <v>39205</v>
+      </c>
+      <c r="K110" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L110" t="n">
+        <v>2122</v>
+      </c>
+      <c r="M110" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>173</v>
+      </c>
+      <c r="P110" t="n">
+        <v>196</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>1243805</v>
+      </c>
+      <c r="R110" t="n">
+        <v>296</v>
+      </c>
+      <c r="S110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-03-02 16:01:22</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>43046</v>
+      </c>
+      <c r="C111" t="n">
+        <v>80714</v>
+      </c>
+      <c r="D111" t="n">
+        <v>14072</v>
+      </c>
+      <c r="E111" t="n">
+        <v>28127</v>
+      </c>
+      <c r="F111" t="n">
+        <v>16675</v>
+      </c>
+      <c r="G111" t="n">
+        <v>50277</v>
+      </c>
+      <c r="H111" t="n">
+        <v>119</v>
+      </c>
+      <c r="I111" t="n">
+        <v>10327</v>
+      </c>
+      <c r="J111" t="n">
+        <v>41820</v>
+      </c>
+      <c r="K111" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L111" t="n">
+        <v>2266</v>
+      </c>
+      <c r="M111" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
+        <v>174</v>
+      </c>
+      <c r="P111" t="n">
+        <v>199</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1316089</v>
+      </c>
+      <c r="R111" t="n">
+        <v>296</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-03-02 16:10:09</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>46670</v>
+      </c>
+      <c r="C112" t="n">
+        <v>84569</v>
+      </c>
+      <c r="D112" t="n">
+        <v>15113</v>
+      </c>
+      <c r="E112" t="n">
+        <v>30125</v>
+      </c>
+      <c r="F112" t="n">
+        <v>17713</v>
+      </c>
+      <c r="G112" t="n">
+        <v>50517</v>
+      </c>
+      <c r="H112" t="n">
+        <v>124</v>
+      </c>
+      <c r="I112" t="n">
+        <v>11309</v>
+      </c>
+      <c r="J112" t="n">
+        <v>43773</v>
+      </c>
+      <c r="K112" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L112" t="n">
+        <v>2468</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" t="n">
+        <v>177</v>
+      </c>
+      <c r="P112" t="n">
+        <v>201</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>1415502</v>
+      </c>
+      <c r="R112" t="n">
+        <v>296</v>
+      </c>
+      <c r="S112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-03-02 16:36:15</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>48559</v>
+      </c>
+      <c r="C113" t="n">
+        <v>85295</v>
+      </c>
+      <c r="D113" t="n">
+        <v>16383</v>
+      </c>
+      <c r="E113" t="n">
+        <v>31940</v>
+      </c>
+      <c r="F113" t="n">
+        <v>18999</v>
+      </c>
+      <c r="G113" t="n">
+        <v>51200</v>
+      </c>
+      <c r="H113" t="n">
+        <v>129</v>
+      </c>
+      <c r="I113" t="n">
+        <v>12168</v>
+      </c>
+      <c r="J113" t="n">
+        <v>46103</v>
+      </c>
+      <c r="K113" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L113" t="n">
+        <v>2776</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>763</v>
+      </c>
+      <c r="O113" t="n">
+        <v>177</v>
+      </c>
+      <c r="P113" t="n">
+        <v>202</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>1441865</v>
+      </c>
+      <c r="R113" t="n">
+        <v>296</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-03-02 16:45:09</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>51228</v>
+      </c>
+      <c r="C114" t="n">
+        <v>89857</v>
+      </c>
+      <c r="D114" t="n">
+        <v>17022</v>
+      </c>
+      <c r="E114" t="n">
+        <v>32826</v>
+      </c>
+      <c r="F114" t="n">
+        <v>19504</v>
+      </c>
+      <c r="G114" t="n">
+        <v>51435</v>
+      </c>
+      <c r="H114" t="n">
+        <v>135</v>
+      </c>
+      <c r="I114" t="n">
+        <v>12467</v>
+      </c>
+      <c r="J114" t="n">
+        <v>46729</v>
+      </c>
+      <c r="K114" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L114" t="n">
+        <v>2776</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>763</v>
+      </c>
+      <c r="O114" t="n">
+        <v>179</v>
+      </c>
+      <c r="P114" t="n">
+        <v>202</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>296</v>
+      </c>
+      <c r="S114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-03-02 23:49:41</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>55008</v>
+      </c>
+      <c r="C115" t="n">
+        <v>93673</v>
+      </c>
+      <c r="D115" t="n">
+        <v>18789</v>
+      </c>
+      <c r="E115" t="n">
+        <v>34021</v>
+      </c>
+      <c r="F115" t="n">
+        <v>21252</v>
+      </c>
+      <c r="G115" t="n">
+        <v>52122</v>
+      </c>
+      <c r="H115" t="n">
+        <v>154</v>
+      </c>
+      <c r="I115" t="n">
+        <v>13222</v>
+      </c>
+      <c r="J115" t="n">
+        <v>48928</v>
+      </c>
+      <c r="K115" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L115" t="n">
+        <v>3064</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" t="n">
+        <v>181</v>
+      </c>
+      <c r="P115" t="n">
+        <v>202</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>1625184</v>
+      </c>
+      <c r="R115" t="n">
+        <v>296</v>
+      </c>
+      <c r="S115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-03-02 23:56:22</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>58018</v>
+      </c>
+      <c r="C116" t="n">
+        <v>97577</v>
+      </c>
+      <c r="D116" t="n">
+        <v>19774</v>
+      </c>
+      <c r="E116" t="n">
+        <v>36282</v>
+      </c>
+      <c r="F116" t="n">
+        <v>22642</v>
+      </c>
+      <c r="G116" t="n">
+        <v>53020</v>
+      </c>
+      <c r="H116" t="n">
+        <v>163</v>
+      </c>
+      <c r="I116" t="n">
+        <v>14021</v>
+      </c>
+      <c r="J116" t="n">
+        <v>51226</v>
+      </c>
+      <c r="K116" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L116" t="n">
+        <v>3197</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="n">
+        <v>181</v>
+      </c>
+      <c r="P116" t="n">
+        <v>205</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>1697909</v>
+      </c>
+      <c r="R116" t="n">
+        <v>296</v>
+      </c>
+      <c r="S116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:28:17</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>62379</v>
+      </c>
+      <c r="C117" t="n">
+        <v>101216</v>
+      </c>
+      <c r="D117" t="n">
+        <v>20598</v>
+      </c>
+      <c r="E117" t="n">
+        <v>38318</v>
+      </c>
+      <c r="F117" t="n">
+        <v>23671</v>
+      </c>
+      <c r="G117" t="n">
+        <v>53522</v>
+      </c>
+      <c r="H117" t="n">
+        <v>180</v>
+      </c>
+      <c r="I117" t="n">
+        <v>14611</v>
+      </c>
+      <c r="J117" t="n">
+        <v>53527</v>
+      </c>
+      <c r="K117" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L117" t="n">
+        <v>3556</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" t="n">
+        <v>982</v>
+      </c>
+      <c r="O117" t="n">
+        <v>183</v>
+      </c>
+      <c r="P117" t="n">
+        <v>208</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R117" t="n">
+        <v>7296</v>
+      </c>
+      <c r="S117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-03-03 00:34:34</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>65930</v>
+      </c>
+      <c r="C118" t="n">
+        <v>104743</v>
+      </c>
+      <c r="D118" t="n">
+        <v>23366</v>
+      </c>
+      <c r="E118" t="n">
+        <v>39434</v>
+      </c>
+      <c r="F118" t="n">
+        <v>26774</v>
+      </c>
+      <c r="G118" t="n">
+        <v>53909</v>
+      </c>
+      <c r="H118" t="n">
+        <v>189</v>
+      </c>
+      <c r="I118" t="n">
+        <v>14919</v>
+      </c>
+      <c r="J118" t="n">
+        <v>55249</v>
+      </c>
+      <c r="K118" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L118" t="n">
+        <v>3707</v>
+      </c>
+      <c r="M118" t="n">
+        <v>0</v>
+      </c>
+      <c r="N118" t="n">
+        <v>1024</v>
+      </c>
+      <c r="O118" t="n">
+        <v>186</v>
+      </c>
+      <c r="P118" t="n">
+        <v>209</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0</v>
+      </c>
+      <c r="R118" t="n">
+        <v>90892</v>
+      </c>
+      <c r="S118" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed memory leak in _grab_region_np
</commit_message>
<xml_diff>
--- a/logs/grind_stats.xlsx
+++ b/logs/grind_stats.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S118"/>
+  <dimension ref="A1:S151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7652,6 +7652,2019 @@
         <v>0</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:45:55</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>70745</v>
+      </c>
+      <c r="C119" t="n">
+        <v>110332</v>
+      </c>
+      <c r="D119" t="n">
+        <v>24326</v>
+      </c>
+      <c r="E119" t="n">
+        <v>41781</v>
+      </c>
+      <c r="F119" t="n">
+        <v>27675</v>
+      </c>
+      <c r="G119" t="n">
+        <v>55139</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" t="n">
+        <v>15450</v>
+      </c>
+      <c r="J119" t="n">
+        <v>57122</v>
+      </c>
+      <c r="K119" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L119" t="n">
+        <v>3857</v>
+      </c>
+      <c r="M119" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="n">
+        <v>186</v>
+      </c>
+      <c r="P119" t="n">
+        <v>210</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R119" t="n">
+        <v>206811</v>
+      </c>
+      <c r="S119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:52:17</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>72611</v>
+      </c>
+      <c r="C120" t="n">
+        <v>114082</v>
+      </c>
+      <c r="D120" t="n">
+        <v>26271</v>
+      </c>
+      <c r="E120" t="n">
+        <v>44351</v>
+      </c>
+      <c r="F120" t="n">
+        <v>29952</v>
+      </c>
+      <c r="G120" t="n">
+        <v>56649</v>
+      </c>
+      <c r="H120" t="n">
+        <v>201</v>
+      </c>
+      <c r="I120" t="n">
+        <v>16199</v>
+      </c>
+      <c r="J120" t="n">
+        <v>59360</v>
+      </c>
+      <c r="K120" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>1164</v>
+      </c>
+      <c r="O120" t="n">
+        <v>190</v>
+      </c>
+      <c r="P120" t="n">
+        <v>211</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R120" t="n">
+        <v>286743</v>
+      </c>
+      <c r="S120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:00:26</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>76137</v>
+      </c>
+      <c r="C121" t="n">
+        <v>118440</v>
+      </c>
+      <c r="D121" t="n">
+        <v>27432</v>
+      </c>
+      <c r="E121" t="n">
+        <v>45279</v>
+      </c>
+      <c r="F121" t="n">
+        <v>30444</v>
+      </c>
+      <c r="G121" t="n">
+        <v>57353</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="n">
+        <v>16988</v>
+      </c>
+      <c r="J121" t="n">
+        <v>61333</v>
+      </c>
+      <c r="K121" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L121" t="n">
+        <v>4228</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="n">
+        <v>196</v>
+      </c>
+      <c r="P121" t="n">
+        <v>212</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0</v>
+      </c>
+      <c r="R121" t="n">
+        <v>390512</v>
+      </c>
+      <c r="S121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:29:37</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>79815</v>
+      </c>
+      <c r="C122" t="n">
+        <v>122629</v>
+      </c>
+      <c r="D122" t="n">
+        <v>28987</v>
+      </c>
+      <c r="E122" t="n">
+        <v>47384</v>
+      </c>
+      <c r="F122" t="n">
+        <v>32084</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="n">
+        <v>213</v>
+      </c>
+      <c r="I122" t="n">
+        <v>17871</v>
+      </c>
+      <c r="J122" t="n">
+        <v>63929</v>
+      </c>
+      <c r="K122" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L122" t="n">
+        <v>4347</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
+        <v>1</v>
+      </c>
+      <c r="O122" t="n">
+        <v>196</v>
+      </c>
+      <c r="P122" t="n">
+        <v>213</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0</v>
+      </c>
+      <c r="R122" t="n">
+        <v>472108</v>
+      </c>
+      <c r="S122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:38:09</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>83156</v>
+      </c>
+      <c r="C123" t="n">
+        <v>126982</v>
+      </c>
+      <c r="D123" t="n">
+        <v>30216</v>
+      </c>
+      <c r="E123" t="n">
+        <v>49313</v>
+      </c>
+      <c r="F123" t="n">
+        <v>33447</v>
+      </c>
+      <c r="G123" t="n">
+        <v>58911</v>
+      </c>
+      <c r="H123" t="n">
+        <v>219</v>
+      </c>
+      <c r="I123" t="n">
+        <v>18609</v>
+      </c>
+      <c r="J123" t="n">
+        <v>66190</v>
+      </c>
+      <c r="K123" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L123" t="n">
+        <v>4406</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>198</v>
+      </c>
+      <c r="P123" t="n">
+        <v>213</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R123" t="n">
+        <v>584166</v>
+      </c>
+      <c r="S123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:09:22</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>86916</v>
+      </c>
+      <c r="C124" t="n">
+        <v>129584</v>
+      </c>
+      <c r="D124" t="n">
+        <v>32134</v>
+      </c>
+      <c r="E124" t="n">
+        <v>50776</v>
+      </c>
+      <c r="F124" t="n">
+        <v>35438</v>
+      </c>
+      <c r="G124" t="n">
+        <v>59127</v>
+      </c>
+      <c r="H124" t="n">
+        <v>225</v>
+      </c>
+      <c r="I124" t="n">
+        <v>19859</v>
+      </c>
+      <c r="J124" t="n">
+        <v>68960</v>
+      </c>
+      <c r="K124" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L124" t="n">
+        <v>4650</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>198</v>
+      </c>
+      <c r="P124" t="n">
+        <v>216</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R124" t="n">
+        <v>677144</v>
+      </c>
+      <c r="S124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:17:24</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>89567</v>
+      </c>
+      <c r="C125" t="n">
+        <v>134007</v>
+      </c>
+      <c r="D125" t="n">
+        <v>33351</v>
+      </c>
+      <c r="E125" t="n">
+        <v>53660</v>
+      </c>
+      <c r="F125" t="n">
+        <v>36958</v>
+      </c>
+      <c r="G125" t="n">
+        <v>59918</v>
+      </c>
+      <c r="H125" t="n">
+        <v>244</v>
+      </c>
+      <c r="I125" t="n">
+        <v>20753</v>
+      </c>
+      <c r="J125" t="n">
+        <v>70719</v>
+      </c>
+      <c r="K125" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L125" t="n">
+        <v>4879</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>200</v>
+      </c>
+      <c r="P125" t="n">
+        <v>218</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R125" t="n">
+        <v>771189</v>
+      </c>
+      <c r="S125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:50:46</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>92917</v>
+      </c>
+      <c r="C126" t="n">
+        <v>137757</v>
+      </c>
+      <c r="D126" t="n">
+        <v>34276</v>
+      </c>
+      <c r="E126" t="n">
+        <v>54886</v>
+      </c>
+      <c r="F126" t="n">
+        <v>38043</v>
+      </c>
+      <c r="G126" t="n">
+        <v>60522</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>21384</v>
+      </c>
+      <c r="J126" t="n">
+        <v>73052</v>
+      </c>
+      <c r="K126" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L126" t="n">
+        <v>4879</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>203</v>
+      </c>
+      <c r="P126" t="n">
+        <v>218</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R126" t="n">
+        <v>871309</v>
+      </c>
+      <c r="S126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:24:59</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>97696</v>
+      </c>
+      <c r="C127" t="n">
+        <v>142337</v>
+      </c>
+      <c r="D127" t="n">
+        <v>35728</v>
+      </c>
+      <c r="E127" t="n">
+        <v>56470</v>
+      </c>
+      <c r="F127" t="n">
+        <v>39960</v>
+      </c>
+      <c r="G127" t="n">
+        <v>61039</v>
+      </c>
+      <c r="H127" t="n">
+        <v>265</v>
+      </c>
+      <c r="I127" t="n">
+        <v>22330</v>
+      </c>
+      <c r="J127" t="n">
+        <v>75295</v>
+      </c>
+      <c r="K127" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L127" t="n">
+        <v>5297</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>204</v>
+      </c>
+      <c r="P127" t="n">
+        <v>220</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R127" t="n">
+        <v>1004466</v>
+      </c>
+      <c r="S127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:18:42</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>102005</v>
+      </c>
+      <c r="C128" t="n">
+        <v>146348</v>
+      </c>
+      <c r="D128" t="n">
+        <v>37868</v>
+      </c>
+      <c r="E128" t="n">
+        <v>59179</v>
+      </c>
+      <c r="F128" t="n">
+        <v>42282</v>
+      </c>
+      <c r="G128" t="n">
+        <v>62103</v>
+      </c>
+      <c r="H128" t="n">
+        <v>270</v>
+      </c>
+      <c r="I128" t="n">
+        <v>23413</v>
+      </c>
+      <c r="J128" t="n">
+        <v>77964</v>
+      </c>
+      <c r="K128" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L128" t="n">
+        <v>5662</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="n">
+        <v>206</v>
+      </c>
+      <c r="P128" t="n">
+        <v>222</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R128" t="n">
+        <v>1098858</v>
+      </c>
+      <c r="S128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:19:52</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>102205</v>
+      </c>
+      <c r="C129" t="n">
+        <v>146348</v>
+      </c>
+      <c r="D129" t="n">
+        <v>40409</v>
+      </c>
+      <c r="E129" t="n">
+        <v>60809</v>
+      </c>
+      <c r="F129" t="n">
+        <v>44410</v>
+      </c>
+      <c r="G129" t="n">
+        <v>62383</v>
+      </c>
+      <c r="H129" t="n">
+        <v>283</v>
+      </c>
+      <c r="I129" t="n">
+        <v>23714</v>
+      </c>
+      <c r="J129" t="n">
+        <v>80213</v>
+      </c>
+      <c r="K129" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L129" t="n">
+        <v>5854</v>
+      </c>
+      <c r="M129" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
+        <v>206</v>
+      </c>
+      <c r="P129" t="n">
+        <v>222</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R129" t="n">
+        <v>1098858</v>
+      </c>
+      <c r="S129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:27:53</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>104454</v>
+      </c>
+      <c r="C130" t="n">
+        <v>150040</v>
+      </c>
+      <c r="D130" t="n">
+        <v>40409</v>
+      </c>
+      <c r="E130" t="n">
+        <v>60809</v>
+      </c>
+      <c r="F130" t="n">
+        <v>44410</v>
+      </c>
+      <c r="G130" t="n">
+        <v>62383</v>
+      </c>
+      <c r="H130" t="n">
+        <v>283</v>
+      </c>
+      <c r="I130" t="n">
+        <v>23714</v>
+      </c>
+      <c r="J130" t="n">
+        <v>80213</v>
+      </c>
+      <c r="K130" t="n">
+        <v>40211</v>
+      </c>
+      <c r="L130" t="n">
+        <v>0</v>
+      </c>
+      <c r="M130" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" t="n">
+        <v>1624</v>
+      </c>
+      <c r="O130" t="n">
+        <v>208</v>
+      </c>
+      <c r="P130" t="n">
+        <v>225</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R130" t="n">
+        <v>1184024</v>
+      </c>
+      <c r="S130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:59:21</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>109366</v>
+      </c>
+      <c r="C131" t="n">
+        <v>154263</v>
+      </c>
+      <c r="D131" t="n">
+        <v>41481</v>
+      </c>
+      <c r="E131" t="n">
+        <v>62091</v>
+      </c>
+      <c r="F131" t="n">
+        <v>45397</v>
+      </c>
+      <c r="G131" t="n">
+        <v>62940</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
+      <c r="I131" t="n">
+        <v>24249</v>
+      </c>
+      <c r="J131" t="n">
+        <v>82238</v>
+      </c>
+      <c r="K131" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L131" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" t="n">
+        <v>1637</v>
+      </c>
+      <c r="O131" t="n">
+        <v>212</v>
+      </c>
+      <c r="P131" t="n">
+        <v>227</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>0</v>
+      </c>
+      <c r="R131" t="n">
+        <v>1289408</v>
+      </c>
+      <c r="S131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-03-03 16:07:18</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>111949</v>
+      </c>
+      <c r="C132" t="n">
+        <v>156928</v>
+      </c>
+      <c r="D132" t="n">
+        <v>43479</v>
+      </c>
+      <c r="E132" t="n">
+        <v>63756</v>
+      </c>
+      <c r="F132" t="n">
+        <v>47292</v>
+      </c>
+      <c r="G132" t="n">
+        <v>63717</v>
+      </c>
+      <c r="H132" t="n">
+        <v>289</v>
+      </c>
+      <c r="I132" t="n">
+        <v>24896</v>
+      </c>
+      <c r="J132" t="n">
+        <v>84618</v>
+      </c>
+      <c r="K132" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L132" t="n">
+        <v>6116</v>
+      </c>
+      <c r="M132" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="n">
+        <v>213</v>
+      </c>
+      <c r="P132" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>0</v>
+      </c>
+      <c r="R132" t="n">
+        <v>1410260</v>
+      </c>
+      <c r="S132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-03-03 16:38:07</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>115164</v>
+      </c>
+      <c r="C133" t="n">
+        <v>160432</v>
+      </c>
+      <c r="D133" t="n">
+        <v>44609</v>
+      </c>
+      <c r="E133" t="n">
+        <v>65631</v>
+      </c>
+      <c r="F133" t="n">
+        <v>48633</v>
+      </c>
+      <c r="G133" t="n">
+        <v>63879</v>
+      </c>
+      <c r="H133" t="n">
+        <v>307</v>
+      </c>
+      <c r="I133" t="n">
+        <v>25646</v>
+      </c>
+      <c r="J133" t="n">
+        <v>86969</v>
+      </c>
+      <c r="K133" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L133" t="n">
+        <v>6236</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" t="n">
+        <v>214</v>
+      </c>
+      <c r="P133" t="n">
+        <v>231</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R133" t="n">
+        <v>1492273</v>
+      </c>
+      <c r="S133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-03-03 17:13:36</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>118959</v>
+      </c>
+      <c r="C134" t="n">
+        <v>165104</v>
+      </c>
+      <c r="D134" t="n">
+        <v>45289</v>
+      </c>
+      <c r="E134" t="n">
+        <v>68097</v>
+      </c>
+      <c r="F134" t="n">
+        <v>49459</v>
+      </c>
+      <c r="G134" t="n">
+        <v>64669</v>
+      </c>
+      <c r="H134" t="n">
+        <v>320</v>
+      </c>
+      <c r="I134" t="n">
+        <v>26228</v>
+      </c>
+      <c r="J134" t="n">
+        <v>88822</v>
+      </c>
+      <c r="K134" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L134" t="n">
+        <v>6507</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+      <c r="O134" t="n">
+        <v>217</v>
+      </c>
+      <c r="P134" t="n">
+        <v>233</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R134" t="n">
+        <v>1614011</v>
+      </c>
+      <c r="S134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-03-03 17:22:31</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>122934</v>
+      </c>
+      <c r="C135" t="n">
+        <v>169230</v>
+      </c>
+      <c r="D135" t="n">
+        <v>47343</v>
+      </c>
+      <c r="E135" t="n">
+        <v>70151</v>
+      </c>
+      <c r="F135" t="n">
+        <v>51551</v>
+      </c>
+      <c r="G135" t="n">
+        <v>65374</v>
+      </c>
+      <c r="H135" t="n">
+        <v>334</v>
+      </c>
+      <c r="I135" t="n">
+        <v>27381</v>
+      </c>
+      <c r="J135" t="n">
+        <v>91301</v>
+      </c>
+      <c r="K135" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L135" t="n">
+        <v>6633</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
+        <v>1842</v>
+      </c>
+      <c r="O135" t="n">
+        <v>223</v>
+      </c>
+      <c r="P135" t="n">
+        <v>234</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R135" t="n">
+        <v>1722649</v>
+      </c>
+      <c r="S135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-03-03 17:25:49</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>123761</v>
+      </c>
+      <c r="C136" t="n">
+        <v>170872</v>
+      </c>
+      <c r="D136" t="n">
+        <v>48871</v>
+      </c>
+      <c r="E136" t="n">
+        <v>71858</v>
+      </c>
+      <c r="F136" t="n">
+        <v>53607</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="n">
+        <v>346</v>
+      </c>
+      <c r="I136" t="n">
+        <v>28106</v>
+      </c>
+      <c r="J136" t="n">
+        <v>93928</v>
+      </c>
+      <c r="K136" t="n">
+        <v>40546</v>
+      </c>
+      <c r="L136" t="n">
+        <v>6832</v>
+      </c>
+      <c r="M136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" t="n">
+        <v>1897</v>
+      </c>
+      <c r="O136" t="n">
+        <v>223</v>
+      </c>
+      <c r="P136" t="n">
+        <v>236</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="R136" t="n">
+        <v>1757002</v>
+      </c>
+      <c r="S136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-03-03 22:22:12</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>2423</v>
+      </c>
+      <c r="C137" t="n">
+        <v>3379</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0</v>
+      </c>
+      <c r="K137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>224</v>
+      </c>
+      <c r="P137" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>0</v>
+      </c>
+      <c r="R137" t="n">
+        <v>1</v>
+      </c>
+      <c r="S137" t="n">
+        <v>67455</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-03-03 22:53:34</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>6060</v>
+      </c>
+      <c r="C138" t="n">
+        <v>6164</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1220</v>
+      </c>
+      <c r="E138" t="n">
+        <v>855</v>
+      </c>
+      <c r="F138" t="n">
+        <v>1328</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="n">
+        <v>19</v>
+      </c>
+      <c r="I138" t="n">
+        <v>768</v>
+      </c>
+      <c r="J138" t="n">
+        <v>1961</v>
+      </c>
+      <c r="K138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" t="n">
+        <v>189</v>
+      </c>
+      <c r="M138" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>224</v>
+      </c>
+      <c r="P138" t="n">
+        <v>241</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>14417</v>
+      </c>
+      <c r="R138" t="n">
+        <v>1</v>
+      </c>
+      <c r="S138" t="n">
+        <v>113281</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-03-03 23:01:13</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>8014</v>
+      </c>
+      <c r="C139" t="n">
+        <v>7939</v>
+      </c>
+      <c r="D139" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E139" t="n">
+        <v>2668</v>
+      </c>
+      <c r="F139" t="n">
+        <v>3169</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="n">
+        <v>31</v>
+      </c>
+      <c r="I139" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J139" t="n">
+        <v>3577</v>
+      </c>
+      <c r="K139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L139" t="n">
+        <v>280</v>
+      </c>
+      <c r="M139" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>225</v>
+      </c>
+      <c r="P139" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>25964</v>
+      </c>
+      <c r="R139" t="n">
+        <v>1</v>
+      </c>
+      <c r="S139" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:23:41</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>11627</v>
+      </c>
+      <c r="C140" t="n">
+        <v>11226</v>
+      </c>
+      <c r="D140" t="n">
+        <v>4033</v>
+      </c>
+      <c r="E140" t="n">
+        <v>4811</v>
+      </c>
+      <c r="F140" t="n">
+        <v>4433</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="n">
+        <v>34</v>
+      </c>
+      <c r="I140" t="n">
+        <v>2122</v>
+      </c>
+      <c r="J140" t="n">
+        <v>5784</v>
+      </c>
+      <c r="K140" t="n">
+        <v>0</v>
+      </c>
+      <c r="L140" t="n">
+        <v>424</v>
+      </c>
+      <c r="M140" t="n">
+        <v>0</v>
+      </c>
+      <c r="N140" t="n">
+        <v>120</v>
+      </c>
+      <c r="O140" t="n">
+        <v>226</v>
+      </c>
+      <c r="P140" t="n">
+        <v>243</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>40420</v>
+      </c>
+      <c r="R140" t="n">
+        <v>1</v>
+      </c>
+      <c r="S140" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:54:51</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>15715</v>
+      </c>
+      <c r="C141" t="n">
+        <v>15882</v>
+      </c>
+      <c r="D141" t="n">
+        <v>5120</v>
+      </c>
+      <c r="E141" t="n">
+        <v>6827</v>
+      </c>
+      <c r="F141" t="n">
+        <v>5665</v>
+      </c>
+      <c r="G141" t="n">
+        <v>2278</v>
+      </c>
+      <c r="H141" t="n">
+        <v>42</v>
+      </c>
+      <c r="I141" t="n">
+        <v>2669</v>
+      </c>
+      <c r="J141" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K141" t="n">
+        <v>0</v>
+      </c>
+      <c r="L141" t="n">
+        <v>500</v>
+      </c>
+      <c r="M141" t="n">
+        <v>0</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>226</v>
+      </c>
+      <c r="P141" t="n">
+        <v>244</v>
+      </c>
+      <c r="Q141" t="n">
+        <v>0</v>
+      </c>
+      <c r="R141" t="n">
+        <v>1</v>
+      </c>
+      <c r="S141" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-03-04 02:02:17</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>17624</v>
+      </c>
+      <c r="C142" t="n">
+        <v>17553</v>
+      </c>
+      <c r="D142" t="n">
+        <v>6572</v>
+      </c>
+      <c r="E142" t="n">
+        <v>8027</v>
+      </c>
+      <c r="F142" t="n">
+        <v>7239</v>
+      </c>
+      <c r="G142" t="n">
+        <v>2857</v>
+      </c>
+      <c r="H142" t="n">
+        <v>42</v>
+      </c>
+      <c r="I142" t="n">
+        <v>3403</v>
+      </c>
+      <c r="J142" t="n">
+        <v>9659</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="n">
+        <v>500</v>
+      </c>
+      <c r="M142" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>229</v>
+      </c>
+      <c r="P142" t="n">
+        <v>245</v>
+      </c>
+      <c r="Q142" t="n">
+        <v>0</v>
+      </c>
+      <c r="R142" t="n">
+        <v>1</v>
+      </c>
+      <c r="S142" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-03-04 12:00:02</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>21933</v>
+      </c>
+      <c r="C143" t="n">
+        <v>23807</v>
+      </c>
+      <c r="D143" t="n">
+        <v>7471</v>
+      </c>
+      <c r="E143" t="n">
+        <v>9377</v>
+      </c>
+      <c r="F143" t="n">
+        <v>8487</v>
+      </c>
+      <c r="G143" t="n">
+        <v>3210</v>
+      </c>
+      <c r="H143" t="n">
+        <v>50</v>
+      </c>
+      <c r="I143" t="n">
+        <v>4044</v>
+      </c>
+      <c r="J143" t="n">
+        <v>11326</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" t="n">
+        <v>683</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>231</v>
+      </c>
+      <c r="P143" t="n">
+        <v>248</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>97592</v>
+      </c>
+      <c r="R143" t="n">
+        <v>1</v>
+      </c>
+      <c r="S143" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-03-04 12:07:45</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>24698</v>
+      </c>
+      <c r="C144" t="n">
+        <v>27943</v>
+      </c>
+      <c r="D144" t="n">
+        <v>8895</v>
+      </c>
+      <c r="E144" t="n">
+        <v>11685</v>
+      </c>
+      <c r="F144" t="n">
+        <v>9799</v>
+      </c>
+      <c r="G144" t="n">
+        <v>4440</v>
+      </c>
+      <c r="H144" t="n">
+        <v>51</v>
+      </c>
+      <c r="I144" t="n">
+        <v>4947</v>
+      </c>
+      <c r="J144" t="n">
+        <v>13828</v>
+      </c>
+      <c r="K144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" t="n">
+        <v>798</v>
+      </c>
+      <c r="M144" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
+        <v>234</v>
+      </c>
+      <c r="P144" t="n">
+        <v>250</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>118124</v>
+      </c>
+      <c r="R144" t="n">
+        <v>1</v>
+      </c>
+      <c r="S144" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-03-04 12:39:18</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>28858</v>
+      </c>
+      <c r="C145" t="n">
+        <v>31791</v>
+      </c>
+      <c r="D145" t="n">
+        <v>9810</v>
+      </c>
+      <c r="E145" t="n">
+        <v>13973</v>
+      </c>
+      <c r="F145" t="n">
+        <v>10805</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="n">
+        <v>52</v>
+      </c>
+      <c r="I145" t="n">
+        <v>5401</v>
+      </c>
+      <c r="J145" t="n">
+        <v>16266</v>
+      </c>
+      <c r="K145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" t="n">
+        <v>1066</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="n">
+        <v>238</v>
+      </c>
+      <c r="P145" t="n">
+        <v>251</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>139081</v>
+      </c>
+      <c r="R145" t="n">
+        <v>1</v>
+      </c>
+      <c r="S145" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-03-04 12:47:15</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>32373</v>
+      </c>
+      <c r="C146" t="n">
+        <v>34631</v>
+      </c>
+      <c r="D146" t="n">
+        <v>11230</v>
+      </c>
+      <c r="E146" t="n">
+        <v>15307</v>
+      </c>
+      <c r="F146" t="n">
+        <v>12425</v>
+      </c>
+      <c r="G146" t="n">
+        <v>6248</v>
+      </c>
+      <c r="H146" t="n">
+        <v>64</v>
+      </c>
+      <c r="I146" t="n">
+        <v>6217</v>
+      </c>
+      <c r="J146" t="n">
+        <v>18276</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="n">
+        <v>1323</v>
+      </c>
+      <c r="M146" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
+        <v>238</v>
+      </c>
+      <c r="P146" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>159360</v>
+      </c>
+      <c r="R146" t="n">
+        <v>1</v>
+      </c>
+      <c r="S146" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-03-04 13:18:50</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>33997</v>
+      </c>
+      <c r="C147" t="n">
+        <v>37275</v>
+      </c>
+      <c r="D147" t="n">
+        <v>13083</v>
+      </c>
+      <c r="E147" t="n">
+        <v>16918</v>
+      </c>
+      <c r="F147" t="n">
+        <v>14380</v>
+      </c>
+      <c r="G147" t="n">
+        <v>6388</v>
+      </c>
+      <c r="H147" t="n">
+        <v>80</v>
+      </c>
+      <c r="I147" t="n">
+        <v>6737</v>
+      </c>
+      <c r="J147" t="n">
+        <v>20545</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" t="n">
+        <v>1572</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
+        <v>443</v>
+      </c>
+      <c r="O147" t="n">
+        <v>244</v>
+      </c>
+      <c r="P147" t="n">
+        <v>253</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>0</v>
+      </c>
+      <c r="R147" t="n">
+        <v>1</v>
+      </c>
+      <c r="S147" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-03-04 13:25:45</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>36776</v>
+      </c>
+      <c r="C148" t="n">
+        <v>40330</v>
+      </c>
+      <c r="D148" t="n">
+        <v>13772</v>
+      </c>
+      <c r="E148" t="n">
+        <v>18983</v>
+      </c>
+      <c r="F148" t="n">
+        <v>15328</v>
+      </c>
+      <c r="G148" t="n">
+        <v>6831</v>
+      </c>
+      <c r="H148" t="n">
+        <v>91</v>
+      </c>
+      <c r="I148" t="n">
+        <v>7532</v>
+      </c>
+      <c r="J148" t="n">
+        <v>22716</v>
+      </c>
+      <c r="K148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" t="n">
+        <v>1855</v>
+      </c>
+      <c r="M148" t="n">
+        <v>0</v>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="n">
+        <v>245</v>
+      </c>
+      <c r="P148" t="n">
+        <v>254</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>0</v>
+      </c>
+      <c r="R148" t="n">
+        <v>1</v>
+      </c>
+      <c r="S148" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-03-04 13:57:34</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>41127</v>
+      </c>
+      <c r="C149" t="n">
+        <v>44354</v>
+      </c>
+      <c r="D149" t="n">
+        <v>14389</v>
+      </c>
+      <c r="E149" t="n">
+        <v>19721</v>
+      </c>
+      <c r="F149" t="n">
+        <v>16135</v>
+      </c>
+      <c r="G149" t="n">
+        <v>7164</v>
+      </c>
+      <c r="H149" t="n">
+        <v>109</v>
+      </c>
+      <c r="I149" t="n">
+        <v>8177</v>
+      </c>
+      <c r="J149" t="n">
+        <v>24378</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
+        <v>1942</v>
+      </c>
+      <c r="M149" t="n">
+        <v>0</v>
+      </c>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="n">
+        <v>248</v>
+      </c>
+      <c r="P149" t="n">
+        <v>255</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>215160</v>
+      </c>
+      <c r="R149" t="n">
+        <v>1</v>
+      </c>
+      <c r="S149" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-03-04 14:07:28</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>44648</v>
+      </c>
+      <c r="C150" t="n">
+        <v>46979</v>
+      </c>
+      <c r="D150" t="n">
+        <v>15626</v>
+      </c>
+      <c r="E150" t="n">
+        <v>21782</v>
+      </c>
+      <c r="F150" t="n">
+        <v>17485</v>
+      </c>
+      <c r="G150" t="n">
+        <v>7590</v>
+      </c>
+      <c r="H150" t="n">
+        <v>114</v>
+      </c>
+      <c r="I150" t="n">
+        <v>8760</v>
+      </c>
+      <c r="J150" t="n">
+        <v>26370</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" t="n">
+        <v>1</v>
+      </c>
+      <c r="O150" t="n">
+        <v>249</v>
+      </c>
+      <c r="P150" t="n">
+        <v>257</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>240122</v>
+      </c>
+      <c r="R150" t="n">
+        <v>1</v>
+      </c>
+      <c r="S150" t="n">
+        <v>143668</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-03-04 14:38:51</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>46569</v>
+      </c>
+      <c r="C151" t="n">
+        <v>49882</v>
+      </c>
+      <c r="D151" t="n">
+        <v>16826</v>
+      </c>
+      <c r="E151" t="n">
+        <v>24073</v>
+      </c>
+      <c r="F151" t="n">
+        <v>18976</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="n">
+        <v>128</v>
+      </c>
+      <c r="I151" t="n">
+        <v>9583</v>
+      </c>
+      <c r="J151" t="n">
+        <v>28706</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
+        <v>2377</v>
+      </c>
+      <c r="M151" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>672</v>
+      </c>
+      <c r="O151" t="n">
+        <v>249</v>
+      </c>
+      <c r="P151" t="n">
+        <v>257</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>255469</v>
+      </c>
+      <c r="R151" t="n">
+        <v>1</v>
+      </c>
+      <c r="S151" t="n">
+        <v>143668</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cleaned up files locations
</commit_message>
<xml_diff>
--- a/logs/grind_stats.xlsx
+++ b/logs/grind_stats.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S151"/>
+  <dimension ref="A1:S176"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9665,6 +9665,1531 @@
         <v>143668</v>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-03-04 23:31:40</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>15389</v>
+      </c>
+      <c r="C152" t="n">
+        <v>15955</v>
+      </c>
+      <c r="D152" t="n">
+        <v>5688</v>
+      </c>
+      <c r="E152" t="n">
+        <v>6809</v>
+      </c>
+      <c r="F152" t="n">
+        <v>6290</v>
+      </c>
+      <c r="G152" t="n">
+        <v>1292</v>
+      </c>
+      <c r="H152" t="n">
+        <v>66</v>
+      </c>
+      <c r="I152" t="n">
+        <v>2672</v>
+      </c>
+      <c r="J152" t="n">
+        <v>8171</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
+        <v>430</v>
+      </c>
+      <c r="M152" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="n">
+        <v>265</v>
+      </c>
+      <c r="P152" t="n">
+        <v>276</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>87528</v>
+      </c>
+      <c r="R152" t="n">
+        <v>0</v>
+      </c>
+      <c r="S152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-03-05 00:01:27</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>18115</v>
+      </c>
+      <c r="C153" t="n">
+        <v>18544</v>
+      </c>
+      <c r="D153" t="n">
+        <v>6838</v>
+      </c>
+      <c r="E153" t="n">
+        <v>8179</v>
+      </c>
+      <c r="F153" t="n">
+        <v>7463</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>72</v>
+      </c>
+      <c r="I153" t="n">
+        <v>3088</v>
+      </c>
+      <c r="J153" t="n">
+        <v>9626</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="n">
+        <v>631</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>268</v>
+      </c>
+      <c r="P153" t="n">
+        <v>277</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>102486</v>
+      </c>
+      <c r="R153" t="n">
+        <v>0</v>
+      </c>
+      <c r="S153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-03-05 00:31:58</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>21055</v>
+      </c>
+      <c r="C154" t="n">
+        <v>21785</v>
+      </c>
+      <c r="D154" t="n">
+        <v>8466</v>
+      </c>
+      <c r="E154" t="n">
+        <v>9172</v>
+      </c>
+      <c r="F154" t="n">
+        <v>8991</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>77</v>
+      </c>
+      <c r="I154" t="n">
+        <v>3712</v>
+      </c>
+      <c r="J154" t="n">
+        <v>11632</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
+        <v>777</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>222</v>
+      </c>
+      <c r="O154" t="n">
+        <v>273</v>
+      </c>
+      <c r="P154" t="n">
+        <v>277</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>120152</v>
+      </c>
+      <c r="R154" t="n">
+        <v>0</v>
+      </c>
+      <c r="S154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:01:02</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>23983</v>
+      </c>
+      <c r="C155" t="n">
+        <v>24927</v>
+      </c>
+      <c r="D155" t="n">
+        <v>9102</v>
+      </c>
+      <c r="E155" t="n">
+        <v>10872</v>
+      </c>
+      <c r="F155" t="n">
+        <v>9961</v>
+      </c>
+      <c r="G155" t="n">
+        <v>2589</v>
+      </c>
+      <c r="H155" t="n">
+        <v>83</v>
+      </c>
+      <c r="I155" t="n">
+        <v>4605</v>
+      </c>
+      <c r="J155" t="n">
+        <v>13887</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
+        <v>903</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>274</v>
+      </c>
+      <c r="P155" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>0</v>
+      </c>
+      <c r="R155" t="n">
+        <v>0</v>
+      </c>
+      <c r="S155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:06:35</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>27033</v>
+      </c>
+      <c r="C156" t="n">
+        <v>26923</v>
+      </c>
+      <c r="D156" t="n">
+        <v>10199</v>
+      </c>
+      <c r="E156" t="n">
+        <v>12253</v>
+      </c>
+      <c r="F156" t="n">
+        <v>11475</v>
+      </c>
+      <c r="G156" t="n">
+        <v>2798</v>
+      </c>
+      <c r="H156" t="n">
+        <v>83</v>
+      </c>
+      <c r="I156" t="n">
+        <v>5111</v>
+      </c>
+      <c r="J156" t="n">
+        <v>15523</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>1018</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>274</v>
+      </c>
+      <c r="P156" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>0</v>
+      </c>
+      <c r="R156" t="n">
+        <v>0</v>
+      </c>
+      <c r="S156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:34:37</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>27982</v>
+      </c>
+      <c r="C157" t="n">
+        <v>29407</v>
+      </c>
+      <c r="D157" t="n">
+        <v>10909</v>
+      </c>
+      <c r="E157" t="n">
+        <v>13540</v>
+      </c>
+      <c r="F157" t="n">
+        <v>12301</v>
+      </c>
+      <c r="G157" t="n">
+        <v>3105</v>
+      </c>
+      <c r="H157" t="n">
+        <v>99</v>
+      </c>
+      <c r="I157" t="n">
+        <v>5723</v>
+      </c>
+      <c r="J157" t="n">
+        <v>16717</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>1092</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>274</v>
+      </c>
+      <c r="P157" t="n">
+        <v>279</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>162982</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0</v>
+      </c>
+      <c r="S157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:41:57</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>30789</v>
+      </c>
+      <c r="C158" t="n">
+        <v>33319</v>
+      </c>
+      <c r="D158" t="n">
+        <v>11721</v>
+      </c>
+      <c r="E158" t="n">
+        <v>14146</v>
+      </c>
+      <c r="F158" t="n">
+        <v>13233</v>
+      </c>
+      <c r="G158" t="n">
+        <v>3473</v>
+      </c>
+      <c r="H158" t="n">
+        <v>109</v>
+      </c>
+      <c r="I158" t="n">
+        <v>6165</v>
+      </c>
+      <c r="J158" t="n">
+        <v>18885</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>1147</v>
+      </c>
+      <c r="M158" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
+        <v>275</v>
+      </c>
+      <c r="P158" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>180680</v>
+      </c>
+      <c r="R158" t="n">
+        <v>0</v>
+      </c>
+      <c r="S158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:11:05</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>34484</v>
+      </c>
+      <c r="C159" t="n">
+        <v>38582</v>
+      </c>
+      <c r="D159" t="n">
+        <v>12687</v>
+      </c>
+      <c r="E159" t="n">
+        <v>15929</v>
+      </c>
+      <c r="F159" t="n">
+        <v>14510</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="n">
+        <v>113</v>
+      </c>
+      <c r="I159" t="n">
+        <v>6971</v>
+      </c>
+      <c r="J159" t="n">
+        <v>20777</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
+        <v>1147</v>
+      </c>
+      <c r="M159" t="n">
+        <v>0</v>
+      </c>
+      <c r="N159" t="n">
+        <v>329</v>
+      </c>
+      <c r="O159" t="n">
+        <v>278</v>
+      </c>
+      <c r="P159" t="n">
+        <v>284</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>198281</v>
+      </c>
+      <c r="R159" t="n">
+        <v>0</v>
+      </c>
+      <c r="S159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:40:04</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>37198</v>
+      </c>
+      <c r="C160" t="n">
+        <v>40928</v>
+      </c>
+      <c r="D160" t="n">
+        <v>14364</v>
+      </c>
+      <c r="E160" t="n">
+        <v>17120</v>
+      </c>
+      <c r="F160" t="n">
+        <v>15988</v>
+      </c>
+      <c r="G160" t="n">
+        <v>4450</v>
+      </c>
+      <c r="H160" t="n">
+        <v>121</v>
+      </c>
+      <c r="I160" t="n">
+        <v>7478</v>
+      </c>
+      <c r="J160" t="n">
+        <v>23204</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>1497</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="n">
+        <v>427</v>
+      </c>
+      <c r="O160" t="n">
+        <v>280</v>
+      </c>
+      <c r="P160" t="n">
+        <v>284</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>216729</v>
+      </c>
+      <c r="R160" t="n">
+        <v>0</v>
+      </c>
+      <c r="S160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:47:20</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>39023</v>
+      </c>
+      <c r="C161" t="n">
+        <v>42939</v>
+      </c>
+      <c r="D161" t="n">
+        <v>15013</v>
+      </c>
+      <c r="E161" t="n">
+        <v>18534</v>
+      </c>
+      <c r="F161" t="n">
+        <v>16685</v>
+      </c>
+      <c r="G161" t="n">
+        <v>4879</v>
+      </c>
+      <c r="H161" t="n">
+        <v>121</v>
+      </c>
+      <c r="I161" t="n">
+        <v>8117</v>
+      </c>
+      <c r="J161" t="n">
+        <v>24857</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>1497</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>282</v>
+      </c>
+      <c r="P161" t="n">
+        <v>286</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>234176</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0</v>
+      </c>
+      <c r="S161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-03-05 03:15:01</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>42957</v>
+      </c>
+      <c r="C162" t="n">
+        <v>47174</v>
+      </c>
+      <c r="D162" t="n">
+        <v>16393</v>
+      </c>
+      <c r="E162" t="n">
+        <v>19660</v>
+      </c>
+      <c r="F162" t="n">
+        <v>18439</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>132</v>
+      </c>
+      <c r="I162" t="n">
+        <v>8858</v>
+      </c>
+      <c r="J162" t="n">
+        <v>26785</v>
+      </c>
+      <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="n">
+        <v>1587</v>
+      </c>
+      <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+      <c r="O162" t="n">
+        <v>283</v>
+      </c>
+      <c r="P162" t="n">
+        <v>288</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>251318</v>
+      </c>
+      <c r="R162" t="n">
+        <v>0</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-03-05 03:43:47</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>44911</v>
+      </c>
+      <c r="C163" t="n">
+        <v>49074</v>
+      </c>
+      <c r="D163" t="n">
+        <v>17706</v>
+      </c>
+      <c r="E163" t="n">
+        <v>21012</v>
+      </c>
+      <c r="F163" t="n">
+        <v>19705</v>
+      </c>
+      <c r="G163" t="n">
+        <v>5449</v>
+      </c>
+      <c r="H163" t="n">
+        <v>136</v>
+      </c>
+      <c r="I163" t="n">
+        <v>9299</v>
+      </c>
+      <c r="J163" t="n">
+        <v>28913</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
+        <v>1864</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+      <c r="O163" t="n">
+        <v>285</v>
+      </c>
+      <c r="P163" t="n">
+        <v>290</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>268082</v>
+      </c>
+      <c r="R163" t="n">
+        <v>0</v>
+      </c>
+      <c r="S163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-03-05 03:51:07</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>49912</v>
+      </c>
+      <c r="C164" t="n">
+        <v>53139</v>
+      </c>
+      <c r="D164" t="n">
+        <v>18729</v>
+      </c>
+      <c r="E164" t="n">
+        <v>23142</v>
+      </c>
+      <c r="F164" t="n">
+        <v>20836</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>139</v>
+      </c>
+      <c r="I164" t="n">
+        <v>9937</v>
+      </c>
+      <c r="J164" t="n">
+        <v>30583</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1992</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="n">
+        <v>0</v>
+      </c>
+      <c r="O164" t="n">
+        <v>287</v>
+      </c>
+      <c r="P164" t="n">
+        <v>291</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>284882</v>
+      </c>
+      <c r="R164" t="n">
+        <v>0</v>
+      </c>
+      <c r="S164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-03-05 04:20:43</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>52262</v>
+      </c>
+      <c r="C165" t="n">
+        <v>55059</v>
+      </c>
+      <c r="D165" t="n">
+        <v>19998</v>
+      </c>
+      <c r="E165" t="n">
+        <v>25058</v>
+      </c>
+      <c r="F165" t="n">
+        <v>22340</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>141</v>
+      </c>
+      <c r="I165" t="n">
+        <v>10237</v>
+      </c>
+      <c r="J165" t="n">
+        <v>32394</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
+        <v>2126</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" t="n">
+        <v>604</v>
+      </c>
+      <c r="O165" t="n">
+        <v>291</v>
+      </c>
+      <c r="P165" t="n">
+        <v>293</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>301881</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-03-05 04:26:45</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>55787</v>
+      </c>
+      <c r="C166" t="n">
+        <v>58730</v>
+      </c>
+      <c r="D166" t="n">
+        <v>20936</v>
+      </c>
+      <c r="E166" t="n">
+        <v>26938</v>
+      </c>
+      <c r="F166" t="n">
+        <v>23680</v>
+      </c>
+      <c r="G166" t="n">
+        <v>7521</v>
+      </c>
+      <c r="H166" t="n">
+        <v>147</v>
+      </c>
+      <c r="I166" t="n">
+        <v>10843</v>
+      </c>
+      <c r="J166" t="n">
+        <v>34202</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="n">
+        <v>2325</v>
+      </c>
+      <c r="M166" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" t="n">
+        <v>659</v>
+      </c>
+      <c r="O166" t="n">
+        <v>292</v>
+      </c>
+      <c r="P166" t="n">
+        <v>294</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>314900</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0</v>
+      </c>
+      <c r="S166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-03-05 04:54:36</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>57019</v>
+      </c>
+      <c r="C167" t="n">
+        <v>62223</v>
+      </c>
+      <c r="D167" t="n">
+        <v>21626</v>
+      </c>
+      <c r="E167" t="n">
+        <v>28317</v>
+      </c>
+      <c r="F167" t="n">
+        <v>24631</v>
+      </c>
+      <c r="G167" t="n">
+        <v>8347</v>
+      </c>
+      <c r="H167" t="n">
+        <v>152</v>
+      </c>
+      <c r="I167" t="n">
+        <v>11304</v>
+      </c>
+      <c r="J167" t="n">
+        <v>36009</v>
+      </c>
+      <c r="K167" t="n">
+        <v>948</v>
+      </c>
+      <c r="L167" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" t="n">
+        <v>0</v>
+      </c>
+      <c r="O167" t="n">
+        <v>293</v>
+      </c>
+      <c r="P167" t="n">
+        <v>294</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>0</v>
+      </c>
+      <c r="R167" t="n">
+        <v>0</v>
+      </c>
+      <c r="S167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-03-05 04:57:24</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>57868</v>
+      </c>
+      <c r="C168" t="n">
+        <v>63407</v>
+      </c>
+      <c r="D168" t="n">
+        <v>22122</v>
+      </c>
+      <c r="E168" t="n">
+        <v>29474</v>
+      </c>
+      <c r="F168" t="n">
+        <v>25133</v>
+      </c>
+      <c r="G168" t="n">
+        <v>10276</v>
+      </c>
+      <c r="H168" t="n">
+        <v>162</v>
+      </c>
+      <c r="I168" t="n">
+        <v>11839</v>
+      </c>
+      <c r="J168" t="n">
+        <v>37460</v>
+      </c>
+      <c r="K168" t="n">
+        <v>1850</v>
+      </c>
+      <c r="L168" t="n">
+        <v>2463</v>
+      </c>
+      <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+      <c r="O168" t="n">
+        <v>293</v>
+      </c>
+      <c r="P168" t="n">
+        <v>295</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>0</v>
+      </c>
+      <c r="R168" t="n">
+        <v>0</v>
+      </c>
+      <c r="S168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-03-05 04:59:54</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>58133</v>
+      </c>
+      <c r="C169" t="n">
+        <v>63672</v>
+      </c>
+      <c r="D169" t="n">
+        <v>22492</v>
+      </c>
+      <c r="E169" t="n">
+        <v>30258</v>
+      </c>
+      <c r="F169" t="n">
+        <v>25425</v>
+      </c>
+      <c r="G169" t="n">
+        <v>11008</v>
+      </c>
+      <c r="H169" t="n">
+        <v>165</v>
+      </c>
+      <c r="I169" t="n">
+        <v>12000</v>
+      </c>
+      <c r="J169" t="n">
+        <v>38013</v>
+      </c>
+      <c r="K169" t="n">
+        <v>2144</v>
+      </c>
+      <c r="L169" t="n">
+        <v>2502</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
+        <v>293</v>
+      </c>
+      <c r="P169" t="n">
+        <v>296</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>0</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:02:14</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>58506</v>
+      </c>
+      <c r="C170" t="n">
+        <v>63780</v>
+      </c>
+      <c r="D170" t="n">
+        <v>22711</v>
+      </c>
+      <c r="E170" t="n">
+        <v>30400</v>
+      </c>
+      <c r="F170" t="n">
+        <v>25654</v>
+      </c>
+      <c r="G170" t="n">
+        <v>11075</v>
+      </c>
+      <c r="H170" t="n">
+        <v>165</v>
+      </c>
+      <c r="I170" t="n">
+        <v>12057</v>
+      </c>
+      <c r="J170" t="n">
+        <v>38418</v>
+      </c>
+      <c r="K170" t="n">
+        <v>2584</v>
+      </c>
+      <c r="L170" t="n">
+        <v>2552</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="n">
+        <v>293</v>
+      </c>
+      <c r="P170" t="n">
+        <v>296</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>0</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0</v>
+      </c>
+      <c r="S170" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:30:42</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>61916</v>
+      </c>
+      <c r="C171" t="n">
+        <v>67709</v>
+      </c>
+      <c r="D171" t="n">
+        <v>22901</v>
+      </c>
+      <c r="E171" t="n">
+        <v>30507</v>
+      </c>
+      <c r="F171" t="n">
+        <v>25897</v>
+      </c>
+      <c r="G171" t="n">
+        <v>11091</v>
+      </c>
+      <c r="H171" t="n">
+        <v>167</v>
+      </c>
+      <c r="I171" t="n">
+        <v>12163</v>
+      </c>
+      <c r="J171" t="n">
+        <v>38536</v>
+      </c>
+      <c r="K171" t="n">
+        <v>2672</v>
+      </c>
+      <c r="L171" t="n">
+        <v>2552</v>
+      </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="n">
+        <v>294</v>
+      </c>
+      <c r="P171" t="n">
+        <v>297</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>350631</v>
+      </c>
+      <c r="R171" t="n">
+        <v>0</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:32:11</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>61916</v>
+      </c>
+      <c r="C172" t="n">
+        <v>67709</v>
+      </c>
+      <c r="D172" t="n">
+        <v>24340</v>
+      </c>
+      <c r="E172" t="n">
+        <v>32248</v>
+      </c>
+      <c r="F172" t="n">
+        <v>27386</v>
+      </c>
+      <c r="G172" t="n">
+        <v>12914</v>
+      </c>
+      <c r="H172" t="n">
+        <v>182</v>
+      </c>
+      <c r="I172" t="n">
+        <v>12756</v>
+      </c>
+      <c r="J172" t="n">
+        <v>40517</v>
+      </c>
+      <c r="K172" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L172" t="n">
+        <v>2625</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
+      <c r="O172" t="n">
+        <v>294</v>
+      </c>
+      <c r="P172" t="n">
+        <v>297</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>350631</v>
+      </c>
+      <c r="R172" t="n">
+        <v>0</v>
+      </c>
+      <c r="S172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:34:38</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>62331</v>
+      </c>
+      <c r="C173" t="n">
+        <v>68172</v>
+      </c>
+      <c r="D173" t="n">
+        <v>24340</v>
+      </c>
+      <c r="E173" t="n">
+        <v>32248</v>
+      </c>
+      <c r="F173" t="n">
+        <v>27386</v>
+      </c>
+      <c r="G173" t="n">
+        <v>12914</v>
+      </c>
+      <c r="H173" t="n">
+        <v>182</v>
+      </c>
+      <c r="I173" t="n">
+        <v>12756</v>
+      </c>
+      <c r="J173" t="n">
+        <v>40517</v>
+      </c>
+      <c r="K173" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L173" t="n">
+        <v>2625</v>
+      </c>
+      <c r="M173" t="n">
+        <v>0</v>
+      </c>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" t="n">
+        <v>294</v>
+      </c>
+      <c r="P173" t="n">
+        <v>297</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>352638</v>
+      </c>
+      <c r="R173" t="n">
+        <v>0</v>
+      </c>
+      <c r="S173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:36:53</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>62621</v>
+      </c>
+      <c r="C174" t="n">
+        <v>69222</v>
+      </c>
+      <c r="D174" t="n">
+        <v>24348</v>
+      </c>
+      <c r="E174" t="n">
+        <v>32849</v>
+      </c>
+      <c r="F174" t="n">
+        <v>27390</v>
+      </c>
+      <c r="G174" t="n">
+        <v>13095</v>
+      </c>
+      <c r="H174" t="n">
+        <v>182</v>
+      </c>
+      <c r="I174" t="n">
+        <v>12796</v>
+      </c>
+      <c r="J174" t="n">
+        <v>40830</v>
+      </c>
+      <c r="K174" t="n">
+        <v>4339</v>
+      </c>
+      <c r="L174" t="n">
+        <v>2625</v>
+      </c>
+      <c r="M174" t="n">
+        <v>0</v>
+      </c>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="n">
+        <v>294</v>
+      </c>
+      <c r="P174" t="n">
+        <v>297</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>354258</v>
+      </c>
+      <c r="R174" t="n">
+        <v>0</v>
+      </c>
+      <c r="S174" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-03-05 05:39:03</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>62664</v>
+      </c>
+      <c r="C175" t="n">
+        <v>69393</v>
+      </c>
+      <c r="D175" t="n">
+        <v>24500</v>
+      </c>
+      <c r="E175" t="n">
+        <v>32893</v>
+      </c>
+      <c r="F175" t="n">
+        <v>27558</v>
+      </c>
+      <c r="G175" t="n">
+        <v>13703</v>
+      </c>
+      <c r="H175" t="n">
+        <v>185</v>
+      </c>
+      <c r="I175" t="n">
+        <v>12824</v>
+      </c>
+      <c r="J175" t="n">
+        <v>41107</v>
+      </c>
+      <c r="K175" t="n">
+        <v>4339</v>
+      </c>
+      <c r="L175" t="n">
+        <v>2671</v>
+      </c>
+      <c r="M175" t="n">
+        <v>0</v>
+      </c>
+      <c r="N175" t="n">
+        <v>0</v>
+      </c>
+      <c r="O175" t="n">
+        <v>294</v>
+      </c>
+      <c r="P175" t="n">
+        <v>298</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>355008</v>
+      </c>
+      <c r="R175" t="n">
+        <v>0</v>
+      </c>
+      <c r="S175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-03-05 06:10:28</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>66025</v>
+      </c>
+      <c r="C176" t="n">
+        <v>74115</v>
+      </c>
+      <c r="D176" t="n">
+        <v>24605</v>
+      </c>
+      <c r="E176" t="n">
+        <v>32912</v>
+      </c>
+      <c r="F176" t="n">
+        <v>27589</v>
+      </c>
+      <c r="G176" t="n">
+        <v>13906</v>
+      </c>
+      <c r="H176" t="n">
+        <v>185</v>
+      </c>
+      <c r="I176" t="n">
+        <v>12862</v>
+      </c>
+      <c r="J176" t="n">
+        <v>41152</v>
+      </c>
+      <c r="K176" t="n">
+        <v>4339</v>
+      </c>
+      <c r="L176" t="n">
+        <v>2671</v>
+      </c>
+      <c r="M176" t="n">
+        <v>0</v>
+      </c>
+      <c r="N176" t="n">
+        <v>756</v>
+      </c>
+      <c r="O176" t="n">
+        <v>297</v>
+      </c>
+      <c r="P176" t="n">
+        <v>298</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>360000</v>
+      </c>
+      <c r="R176" t="n">
+        <v>20569</v>
+      </c>
+      <c r="S176" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added logic for multiple poly vaults
</commit_message>
<xml_diff>
--- a/logs/grind_stats.xlsx
+++ b/logs/grind_stats.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S176"/>
+  <dimension ref="A1:S177"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -11190,6 +11190,67 @@
         <v>0</v>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-03-05 07:49:41</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>75183</v>
+      </c>
+      <c r="C177" t="n">
+        <v>83452</v>
+      </c>
+      <c r="D177" t="n">
+        <v>28315</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>32147</v>
+      </c>
+      <c r="G177" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H177" t="n">
+        <v>219</v>
+      </c>
+      <c r="I177" t="n">
+        <v>14589</v>
+      </c>
+      <c r="J177" t="n">
+        <v>47739</v>
+      </c>
+      <c r="K177" t="n">
+        <v>5216</v>
+      </c>
+      <c r="L177" t="n">
+        <v>3473</v>
+      </c>
+      <c r="M177" t="n">
+        <v>0</v>
+      </c>
+      <c r="N177" t="n">
+        <v>0</v>
+      </c>
+      <c r="O177" t="n">
+        <v>300</v>
+      </c>
+      <c r="P177" t="n">
+        <v>302</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>360000</v>
+      </c>
+      <c r="R177" t="n">
+        <v>73202</v>
+      </c>
+      <c r="S177" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>